<commit_message>
fix(excel): preservacao do logo da codisplan e preenchimento da data de entrada
</commit_message>
<xml_diff>
--- a/storage/templates/modelo_padrao_antecipacao_parcial.xlsx
+++ b/storage/templates/modelo_padrao_antecipacao_parcial.xlsx
@@ -620,6 +620,96 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1771650" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1771650" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1771650" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
@@ -929,6 +1019,66 @@
     </pic>
     <clientData/>
   </twoCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1771650" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1771650" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -5612,6 +5762,7 @@
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" scale="77" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7810,6 +7961,7 @@
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" scale="77" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -10008,6 +10160,7 @@
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" scale="77" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -25406,6 +25559,7 @@
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" scale="77" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -27604,5 +27758,6 @@
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="9" scale="77" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>